<commit_message>
docs(bom): ajoute alimentation 12V manquante au BOM canonique
- BOM_v4_secteur.xlsx: +1 ligne 'Alimentation 12V 2A (×2)' (pompes 12V),
  renumérotation 1->44, recalcul totaux: 214,40€ + 15% = 246,56€
- Câblage déjà complet (Wago 221, JST, câble silicone, gaine, serre-câbles)
- CLAUDE.md + sourcing_consolidation_v4.md: prix/nb lignes alignés (44 / 246,56€)
</commit_message>
<xml_diff>
--- a/docs/BOM_v4_secteur.xlsx
+++ b/docs/BOM_v4_secteur.xlsx
@@ -660,7 +660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="26" min="1" max="1"/>
@@ -949,36 +949,36 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="27">
-      <c r="A12" s="34" t="n">
+      <c r="A12" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="35" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>MCU &amp; ÉLECTRONIQUE</t>
         </is>
       </c>
-      <c r="C12" s="35" t="inlineStr">
-        <is>
-          <t>Module LED RGB KY-016 (×2)</t>
-        </is>
-      </c>
-      <c r="D12" s="36" t="inlineStr">
-        <is>
-          <t>Cathode commune, résistances intégrées (3 GPIO PWM). 1 maître + 1 esclave</t>
-        </is>
-      </c>
-      <c r="E12" s="34" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Alimentation 12V 2A (×2)</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Bloc secteur dédié pompe. Maître: pompe B. Esclave: pompe A. ⚠ AJOUT (pompes 12V)</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="37" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G12" s="38" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="H12" s="39" t="inlineStr">
-        <is>
-          <t>AliExpress (lot 10)</t>
+      <c r="F12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>10</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Amazon.fr</t>
         </is>
       </c>
     </row>
@@ -993,26 +993,26 @@
       </c>
       <c r="C13" s="35" t="inlineStr">
         <is>
-          <t>Résistances 220Ω (LED RGB)</t>
+          <t>Module LED RGB KY-016 (×2)</t>
         </is>
       </c>
       <c r="D13" s="36" t="inlineStr">
         <is>
-          <t>Intégrées au module KY-016 — non requises</t>
+          <t>Cathode commune, résistances intégrées (3 GPIO PWM). 1 maître + 1 esclave</t>
         </is>
       </c>
       <c r="E13" s="34" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F13" s="37" t="n">
-        <v>0.1</v>
+        <v>0.8</v>
       </c>
       <c r="G13" s="38" t="n">
-        <v>0</v>
+        <v>1.6</v>
       </c>
       <c r="H13" s="39" t="inlineStr">
         <is>
-          <t>AliExpress (lot 100)</t>
+          <t>AliExpress (lot 10)</t>
         </is>
       </c>
     </row>
@@ -1027,22 +1027,22 @@
       </c>
       <c r="C14" s="35" t="inlineStr">
         <is>
-          <t>Résistance 10kΩ (pull-down MOSFET)</t>
+          <t>Résistances 220Ω (LED RGB)</t>
         </is>
       </c>
       <c r="D14" s="36" t="inlineStr">
         <is>
-          <t>Pompe OFF si MCU crash. 1 par zone</t>
+          <t>Intégrées au module KY-016 — non requises</t>
         </is>
       </c>
       <c r="E14" s="34" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F14" s="37" t="n">
         <v>0.1</v>
       </c>
       <c r="G14" s="38" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="H14" s="39" t="inlineStr">
         <is>
@@ -1061,22 +1061,22 @@
       </c>
       <c r="C15" s="35" t="inlineStr">
         <is>
-          <t>Résistance 4.7kΩ (pull-up I2C)</t>
+          <t>Résistance 10kΩ (pull-down MOSFET)</t>
         </is>
       </c>
       <c r="D15" s="36" t="inlineStr">
         <is>
-          <t>SDA + SCL, 1 paire par ESP32</t>
+          <t>Pompe OFF si MCU crash. 1 par zone</t>
         </is>
       </c>
       <c r="E15" s="34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F15" s="37" t="n">
         <v>0.1</v>
       </c>
       <c r="G15" s="38" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="H15" s="39" t="inlineStr">
         <is>
@@ -1095,26 +1095,26 @@
       </c>
       <c r="C16" s="35" t="inlineStr">
         <is>
-          <t>Condensateur 100µF 25V</t>
+          <t>Résistance 4.7kΩ (pull-up I2C)</t>
         </is>
       </c>
       <c r="D16" s="36" t="inlineStr">
         <is>
-          <t>Filtrage entrée USB</t>
+          <t>SDA + SCL, 1 paire par ESP32</t>
         </is>
       </c>
       <c r="E16" s="34" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F16" s="37" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G16" s="38" t="n">
         <v>0.4</v>
       </c>
       <c r="H16" s="39" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>AliExpress (lot 100)</t>
         </is>
       </c>
     </row>
@@ -1127,94 +1127,94 @@
           <t>MCU &amp; ÉLECTRONIQUE</t>
         </is>
       </c>
-      <c r="C17" s="40" t="inlineStr">
+      <c r="C17" s="35" t="inlineStr">
+        <is>
+          <t>Condensateur 100µF 25V</t>
+        </is>
+      </c>
+      <c r="D17" s="36" t="inlineStr">
+        <is>
+          <t>Filtrage entrée USB</t>
+        </is>
+      </c>
+      <c r="E17" s="34" t="n">
+        <v>2</v>
+      </c>
+      <c r="F17" s="37" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G17" s="38" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="H17" s="39" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1" s="27">
+      <c r="A18" s="34" t="n">
+        <v>13</v>
+      </c>
+      <c r="B18" s="35" t="inlineStr">
+        <is>
+          <t>MCU &amp; ÉLECTRONIQUE</t>
+        </is>
+      </c>
+      <c r="C18" s="40" t="inlineStr">
         <is>
           <t>Fusible 3A + porte-fusible inline</t>
         </is>
       </c>
-      <c r="D17" s="36" t="inlineStr">
+      <c r="D18" s="36" t="inlineStr">
         <is>
           <t>Sur ligne 12V pompe esclave (si pompe 12V)</t>
         </is>
       </c>
-      <c r="E17" s="34" t="n">
+      <c r="E18" s="34" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="37" t="n">
+      <c r="F18" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="38" t="n">
+      <c r="G18" s="38" t="n">
         <v>2</v>
       </c>
-      <c r="H17" s="39" t="inlineStr">
+      <c r="H18" s="39" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="27">
-      <c r="A18" s="41" t="inlineStr">
+    <row r="19" ht="15" customHeight="1" s="27">
+      <c r="A19" s="41" t="inlineStr">
         <is>
           <t>Sous-total MCU &amp; ÉLECTRONIQUE</t>
-        </is>
-      </c>
-      <c r="B18" s="32" t="n"/>
-      <c r="C18" s="32" t="n"/>
-      <c r="D18" s="32" t="n"/>
-      <c r="E18" s="32" t="n"/>
-      <c r="F18" s="33" t="n"/>
-      <c r="G18" s="42" t="n">
-        <v>50.6</v>
-      </c>
-      <c r="H18" s="43" t="n"/>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="27">
-      <c r="A19" s="31" t="inlineStr">
-        <is>
-          <t>📡 CAPTEURS</t>
         </is>
       </c>
       <c r="B19" s="32" t="n"/>
       <c r="C19" s="32" t="n"/>
       <c r="D19" s="32" t="n"/>
       <c r="E19" s="32" t="n"/>
-      <c r="F19" s="32" t="n"/>
-      <c r="G19" s="32" t="n"/>
-      <c r="H19" s="33" t="n"/>
+      <c r="F19" s="33" t="n"/>
+      <c r="G19" s="42" t="n">
+        <v>60.6</v>
+      </c>
+      <c r="H19" s="43" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="27">
-      <c r="A20" s="34" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="35" t="inlineStr">
-        <is>
-          <t>CAPTEURS</t>
-        </is>
-      </c>
-      <c r="C20" s="35" t="inlineStr">
-        <is>
-          <t>Capteur humidité capacitif v1.2</t>
-        </is>
-      </c>
-      <c r="D20" s="36" t="inlineStr">
-        <is>
-          <t>Analogique 3.3-5V (puce TLC555), JST 3 pins. v1.2 (pas v2.0). Tester chaque unité. 10 par zone</t>
-        </is>
-      </c>
-      <c r="E20" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="F20" s="37" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="G20" s="38" t="n">
-        <v>16</v>
-      </c>
-      <c r="H20" s="39" t="inlineStr">
-        <is>
-          <t>AliExpress (lot 10 ~8€)</t>
-        </is>
-      </c>
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>📡 CAPTEURS</t>
+        </is>
+      </c>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="32" t="n"/>
+      <c r="F20" s="32" t="n"/>
+      <c r="G20" s="32" t="n"/>
+      <c r="H20" s="33" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="27">
       <c r="A21" s="34" t="n">
@@ -1227,26 +1227,26 @@
       </c>
       <c r="C21" s="35" t="inlineStr">
         <is>
-          <t>Capteur US étanche JSN-SR04T</t>
+          <t>Capteur humidité capacitif v1.2</t>
         </is>
       </c>
       <c r="D21" s="36" t="inlineStr">
         <is>
-          <t>IP67, sonde déportée. 1 par zone/réservoir</t>
+          <t>Analogique 3.3-5V (puce TLC555), JST 3 pins. v1.2 (pas v2.0). Tester chaque unité. 10 par zone</t>
         </is>
       </c>
       <c r="E21" s="34" t="n">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="F21" s="37" t="n">
-        <v>4.5</v>
+        <v>0.8</v>
       </c>
       <c r="G21" s="38" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="H21" s="39" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>AliExpress (lot 10 ~8€)</t>
         </is>
       </c>
     </row>
@@ -1261,22 +1261,22 @@
       </c>
       <c r="C22" s="35" t="inlineStr">
         <is>
-          <t>Capteur BME280 breakout I2C</t>
+          <t>Capteur US étanche JSN-SR04T</t>
         </is>
       </c>
       <c r="D22" s="36" t="inlineStr">
         <is>
-          <t>T°/HR/P extérieur. Esclave balcon uniquement</t>
+          <t>IP67, sonde déportée. 1 par zone/réservoir</t>
         </is>
       </c>
       <c r="E22" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F22" s="37" t="n">
-        <v>2.5</v>
+        <v>4.5</v>
       </c>
       <c r="G22" s="38" t="n">
-        <v>2.5</v>
+        <v>9</v>
       </c>
       <c r="H22" s="39" t="inlineStr">
         <is>
@@ -1295,12 +1295,12 @@
       </c>
       <c r="C23" s="35" t="inlineStr">
         <is>
-          <t>Module RTC DS3231 + pile CR2032</t>
+          <t>Capteur BME280 breakout I2C</t>
         </is>
       </c>
       <c r="D23" s="36" t="inlineStr">
         <is>
-          <t>I2C 0x68. Horloge maître uniquement</t>
+          <t>T°/HR/P extérieur. Esclave balcon uniquement</t>
         </is>
       </c>
       <c r="E23" s="34" t="n">
@@ -1329,22 +1329,22 @@
       </c>
       <c r="C24" s="35" t="inlineStr">
         <is>
-          <t>LCD TFT 2.4" ILI9341 + tactile</t>
+          <t>Module RTC DS3231 + pile CR2032</t>
         </is>
       </c>
       <c r="D24" s="36" t="inlineStr">
         <is>
-          <t>320×240 SPI + XPT2046. Dashboard maître</t>
+          <t>I2C 0x68. Horloge maître uniquement</t>
         </is>
       </c>
       <c r="E24" s="34" t="n">
         <v>1</v>
       </c>
       <c r="F24" s="37" t="n">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>6</v>
+        <v>2.5</v>
       </c>
       <c r="H24" s="39" t="inlineStr">
         <is>
@@ -1363,92 +1363,92 @@
       </c>
       <c r="C25" s="35" t="inlineStr">
         <is>
-          <t>Capteur INA219 breakout I2C</t>
+          <t>LCD TFT 2.4" ILI9341 + tactile</t>
         </is>
       </c>
       <c r="D25" s="36" t="inlineStr">
         <is>
-          <t>Courant pompe A. Esclave uniquement</t>
+          <t>320×240 SPI + XPT2046. Dashboard maître</t>
         </is>
       </c>
       <c r="E25" s="34" t="n">
         <v>1</v>
       </c>
       <c r="F25" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="G25" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="H25" s="39" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1" s="27">
+      <c r="A26" s="34" t="n">
+        <v>19</v>
+      </c>
+      <c r="B26" s="35" t="inlineStr">
+        <is>
+          <t>CAPTEURS</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="inlineStr">
+        <is>
+          <t>Capteur INA219 breakout I2C</t>
+        </is>
+      </c>
+      <c r="D26" s="36" t="inlineStr">
+        <is>
+          <t>Courant pompe A. Esclave uniquement</t>
+        </is>
+      </c>
+      <c r="E26" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="38" t="n">
+      <c r="G26" s="38" t="n">
         <v>2</v>
       </c>
-      <c r="H25" s="39" t="inlineStr">
+      <c r="H26" s="39" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="27">
-      <c r="A26" s="41" t="inlineStr">
+    <row r="27" ht="15" customHeight="1" s="27">
+      <c r="A27" s="41" t="inlineStr">
         <is>
           <t>Sous-total CAPTEURS</t>
-        </is>
-      </c>
-      <c r="B26" s="32" t="n"/>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="32" t="n"/>
-      <c r="F26" s="33" t="n"/>
-      <c r="G26" s="42" t="n">
-        <v>38</v>
-      </c>
-      <c r="H26" s="43" t="n"/>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="27">
-      <c r="A27" s="31" t="inlineStr">
-        <is>
-          <t>💧 HYDRAULIQUE</t>
         </is>
       </c>
       <c r="B27" s="32" t="n"/>
       <c r="C27" s="32" t="n"/>
       <c r="D27" s="32" t="n"/>
       <c r="E27" s="32" t="n"/>
-      <c r="F27" s="32" t="n"/>
-      <c r="G27" s="32" t="n"/>
-      <c r="H27" s="33" t="n"/>
+      <c r="F27" s="33" t="n"/>
+      <c r="G27" s="42" t="n">
+        <v>38</v>
+      </c>
+      <c r="H27" s="43" t="n"/>
     </row>
     <row r="28" ht="15" customHeight="1" s="27">
-      <c r="A28" s="34" t="n">
-        <v>19</v>
-      </c>
-      <c r="B28" s="35" t="inlineStr">
-        <is>
-          <t>HYDRAULIQUE</t>
-        </is>
-      </c>
-      <c r="C28" s="44" t="inlineStr">
-        <is>
-          <t>Réservoirs 25L (EXISTANTS)</t>
-        </is>
-      </c>
-      <c r="D28" s="36" t="inlineStr">
-        <is>
-          <t>2× balcon (50L) + 1× intérieur (25L)</t>
-        </is>
-      </c>
-      <c r="E28" s="34" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" s="37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="39" t="inlineStr">
-        <is>
-          <t>EXISTANT</t>
-        </is>
-      </c>
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>💧 HYDRAULIQUE</t>
+        </is>
+      </c>
+      <c r="B28" s="32" t="n"/>
+      <c r="C28" s="32" t="n"/>
+      <c r="D28" s="32" t="n"/>
+      <c r="E28" s="32" t="n"/>
+      <c r="F28" s="32" t="n"/>
+      <c r="G28" s="32" t="n"/>
+      <c r="H28" s="33" t="n"/>
     </row>
     <row r="29" ht="15" customHeight="1" s="27">
       <c r="A29" s="34" t="n">
@@ -1459,28 +1459,28 @@
           <t>HYDRAULIQUE</t>
         </is>
       </c>
-      <c r="C29" s="35" t="inlineStr">
-        <is>
-          <t>Pompe péristaltique 12V (×2 zones)</t>
+      <c r="C29" s="44" t="inlineStr">
+        <is>
+          <t>Réservoirs 25L (EXISTANTS)</t>
         </is>
       </c>
       <c r="D29" s="36" t="inlineStr">
         <is>
-          <t>Auto-amorçante, silicone. 1 par zone</t>
+          <t>2× balcon (50L) + 1× intérieur (25L)</t>
         </is>
       </c>
       <c r="E29" s="34" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F29" s="37" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G29" s="38" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H29" s="39" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>EXISTANT</t>
         </is>
       </c>
     </row>
@@ -1495,26 +1495,26 @@
       </c>
       <c r="C30" s="35" t="inlineStr">
         <is>
-          <t>Passe-cloison PVC 1/2" + joints EPDM</t>
+          <t>Pompe péristaltique 12V (×2 zones)</t>
         </is>
       </c>
       <c r="D30" s="36" t="inlineStr">
         <is>
-          <t>Inter-bidon balcon uniquement</t>
+          <t>Auto-amorçante, silicone. 1 par zone</t>
         </is>
       </c>
       <c r="E30" s="34" t="n">
         <v>2</v>
       </c>
       <c r="F30" s="37" t="n">
-        <v>1.5</v>
+        <v>5</v>
       </c>
       <c r="G30" s="38" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="H30" s="39" t="inlineStr">
         <is>
-          <t>Leroy Merlin</t>
+          <t>AliExpress</t>
         </is>
       </c>
     </row>
@@ -1529,19 +1529,19 @@
       </c>
       <c r="C31" s="35" t="inlineStr">
         <is>
-          <t>Tube tressé renforcé 1/2"</t>
+          <t>Passe-cloison PVC 1/2" + joints EPDM</t>
         </is>
       </c>
       <c r="D31" s="36" t="inlineStr">
         <is>
-          <t>30cm inter-bidon balcon</t>
+          <t>Inter-bidon balcon uniquement</t>
         </is>
       </c>
       <c r="E31" s="34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F31" s="37" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="G31" s="38" t="n">
         <v>3</v>
@@ -1563,12 +1563,12 @@
       </c>
       <c r="C32" s="35" t="inlineStr">
         <is>
-          <t>Téflon PTFE + colliers inox 1/2"</t>
+          <t>Tube tressé renforcé 1/2"</t>
         </is>
       </c>
       <c r="D32" s="36" t="inlineStr">
         <is>
-          <t>Étanchéité raccords</t>
+          <t>30cm inter-bidon balcon</t>
         </is>
       </c>
       <c r="E32" s="34" t="n">
@@ -1582,7 +1582,7 @@
       </c>
       <c r="H32" s="39" t="inlineStr">
         <is>
-          <t>Bricomarché</t>
+          <t>Leroy Merlin</t>
         </is>
       </c>
     </row>
@@ -1597,26 +1597,26 @@
       </c>
       <c r="C33" s="35" t="inlineStr">
         <is>
-          <t>Tube silicone/PVC 4/6mm</t>
+          <t>Téflon PTFE + colliers inox 1/2"</t>
         </is>
       </c>
       <c r="D33" s="36" t="inlineStr">
         <is>
-          <t>Rouleau 20m. Distribution goutteurs</t>
+          <t>Étanchéité raccords</t>
         </is>
       </c>
       <c r="E33" s="34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F33" s="37" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G33" s="38" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="H33" s="39" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>Bricomarché</t>
         </is>
       </c>
     </row>
@@ -1631,19 +1631,19 @@
       </c>
       <c r="C34" s="35" t="inlineStr">
         <is>
-          <t>Goutteurs auto-compensants (mix)</t>
+          <t>Tube silicone/PVC 4/6mm</t>
         </is>
       </c>
       <c r="D34" s="36" t="inlineStr">
         <is>
-          <t>CNL: 10× 2L/h + 6× 4L/h + 4× 8L/h</t>
+          <t>Rouleau 20m. Distribution goutteurs</t>
         </is>
       </c>
       <c r="E34" s="34" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="F34" s="37" t="n">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="G34" s="38" t="n">
         <v>10</v>
@@ -1665,26 +1665,26 @@
       </c>
       <c r="C35" s="35" t="inlineStr">
         <is>
-          <t>Connecteurs T / Y 4mm</t>
+          <t>Goutteurs auto-compensants (mix)</t>
         </is>
       </c>
       <c r="D35" s="36" t="inlineStr">
         <is>
-          <t>Dérivation réseau tubes</t>
+          <t>CNL: 10× 2L/h + 6× 4L/h + 4× 8L/h</t>
         </is>
       </c>
       <c r="E35" s="34" t="n">
         <v>20</v>
       </c>
       <c r="F35" s="37" t="n">
-        <v>0.2</v>
+        <v>0.5</v>
       </c>
       <c r="G35" s="38" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="H35" s="39" t="inlineStr">
         <is>
-          <t>AliExpress (lot 50)</t>
+          <t>AliExpress</t>
         </is>
       </c>
     </row>
@@ -1699,92 +1699,92 @@
       </c>
       <c r="C36" s="35" t="inlineStr">
         <is>
+          <t>Connecteurs T / Y 4mm</t>
+        </is>
+      </c>
+      <c r="D36" s="36" t="inlineStr">
+        <is>
+          <t>Dérivation réseau tubes</t>
+        </is>
+      </c>
+      <c r="E36" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="F36" s="37" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G36" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="H36" s="39" t="inlineStr">
+        <is>
+          <t>AliExpress (lot 50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="15" customHeight="1" s="27">
+      <c r="A37" s="34" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" s="35" t="inlineStr">
+        <is>
+          <t>HYDRAULIQUE</t>
+        </is>
+      </c>
+      <c r="C37" s="35" t="inlineStr">
+        <is>
           <t>Colliers de serrage 6mm inox</t>
         </is>
       </c>
-      <c r="D36" s="36" t="inlineStr">
+      <c r="D37" s="36" t="inlineStr">
         <is>
           <t>Fixation tubes</t>
         </is>
       </c>
-      <c r="E36" s="34" t="n">
+      <c r="E37" s="34" t="n">
         <v>30</v>
       </c>
-      <c r="F36" s="37" t="n">
+      <c r="F37" s="37" t="n">
         <v>0.1</v>
       </c>
-      <c r="G36" s="38" t="n">
+      <c r="G37" s="38" t="n">
         <v>3</v>
       </c>
-      <c r="H36" s="39" t="inlineStr">
+      <c r="H37" s="39" t="inlineStr">
         <is>
           <t>AliExpress (lot 100)</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="27">
-      <c r="A37" s="41" t="inlineStr">
+    <row r="38" ht="15" customHeight="1" s="27">
+      <c r="A38" s="41" t="inlineStr">
         <is>
           <t>Sous-total HYDRAULIQUE</t>
-        </is>
-      </c>
-      <c r="B37" s="32" t="n"/>
-      <c r="C37" s="32" t="n"/>
-      <c r="D37" s="32" t="n"/>
-      <c r="E37" s="32" t="n"/>
-      <c r="F37" s="33" t="n"/>
-      <c r="G37" s="42" t="n">
-        <v>46</v>
-      </c>
-      <c r="H37" s="43" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="27">
-      <c r="A38" s="31" t="inlineStr">
-        <is>
-          <t>🔧 CÂBLAGE PLUG-AND-PLAY</t>
         </is>
       </c>
       <c r="B38" s="32" t="n"/>
       <c r="C38" s="32" t="n"/>
       <c r="D38" s="32" t="n"/>
       <c r="E38" s="32" t="n"/>
-      <c r="F38" s="32" t="n"/>
-      <c r="G38" s="32" t="n"/>
-      <c r="H38" s="33" t="n"/>
+      <c r="F38" s="33" t="n"/>
+      <c r="G38" s="42" t="n">
+        <v>46</v>
+      </c>
+      <c r="H38" s="43" t="n"/>
     </row>
     <row r="39" ht="15" customHeight="1" s="27">
-      <c r="A39" s="34" t="n">
-        <v>28</v>
-      </c>
-      <c r="B39" s="35" t="inlineStr">
-        <is>
-          <t>CÂBLAGE PLUG-AND-PLAY</t>
-        </is>
-      </c>
-      <c r="C39" s="35" t="inlineStr">
-        <is>
-          <t>Wago 221-412 (2 entrées)</t>
-        </is>
-      </c>
-      <c r="D39" s="36" t="inlineStr">
-        <is>
-          <t>Connexion rapide 12-24 AWG</t>
-        </is>
-      </c>
-      <c r="E39" s="34" t="n">
-        <v>10</v>
-      </c>
-      <c r="F39" s="37" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="G39" s="38" t="n">
-        <v>5</v>
-      </c>
-      <c r="H39" s="39" t="inlineStr">
-        <is>
-          <t>Leroy Merlin</t>
-        </is>
-      </c>
+      <c r="A39" s="31" t="inlineStr">
+        <is>
+          <t>🔧 CÂBLAGE PLUG-AND-PLAY</t>
+        </is>
+      </c>
+      <c r="B39" s="32" t="n"/>
+      <c r="C39" s="32" t="n"/>
+      <c r="D39" s="32" t="n"/>
+      <c r="E39" s="32" t="n"/>
+      <c r="F39" s="32" t="n"/>
+      <c r="G39" s="32" t="n"/>
+      <c r="H39" s="33" t="n"/>
     </row>
     <row r="40" ht="15" customHeight="1" s="27">
       <c r="A40" s="34" t="n">
@@ -1797,22 +1797,22 @@
       </c>
       <c r="C40" s="35" t="inlineStr">
         <is>
-          <t>Wago 221-413 (3 entrées)</t>
+          <t>Wago 221-412 (2 entrées)</t>
         </is>
       </c>
       <c r="D40" s="36" t="inlineStr">
         <is>
-          <t>Jonction 3.3V/GND/Signal</t>
+          <t>Connexion rapide 12-24 AWG</t>
         </is>
       </c>
       <c r="E40" s="34" t="n">
         <v>10</v>
       </c>
       <c r="F40" s="37" t="n">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="G40" s="38" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H40" s="39" t="inlineStr">
         <is>
@@ -1831,22 +1831,22 @@
       </c>
       <c r="C41" s="35" t="inlineStr">
         <is>
-          <t>Wago 221-415 (5 entrées)</t>
+          <t>Wago 221-413 (3 entrées)</t>
         </is>
       </c>
       <c r="D41" s="36" t="inlineStr">
         <is>
-          <t>Distribution rails</t>
+          <t>Jonction 3.3V/GND/Signal</t>
         </is>
       </c>
       <c r="E41" s="34" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F41" s="37" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G41" s="38" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H41" s="39" t="inlineStr">
         <is>
@@ -1865,26 +1865,26 @@
       </c>
       <c r="C42" s="35" t="inlineStr">
         <is>
-          <t>Câble silicone 22AWG rouge+noir</t>
+          <t>Wago 221-415 (5 entrées)</t>
         </is>
       </c>
       <c r="D42" s="36" t="inlineStr">
         <is>
-          <t>5m chaque, signal</t>
+          <t>Distribution rails</t>
         </is>
       </c>
       <c r="E42" s="34" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F42" s="37" t="n">
-        <v>4</v>
+        <v>0.8</v>
       </c>
       <c r="G42" s="38" t="n">
         <v>4</v>
       </c>
       <c r="H42" s="39" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>Leroy Merlin</t>
         </is>
       </c>
     </row>
@@ -1899,26 +1899,26 @@
       </c>
       <c r="C43" s="35" t="inlineStr">
         <is>
-          <t>Câbles Dupont F-F 20cm</t>
+          <t>Câble silicone 22AWG rouge+noir</t>
         </is>
       </c>
       <c r="D43" s="36" t="inlineStr">
         <is>
-          <t>MUX ↔ breakout</t>
+          <t>5m chaque, signal</t>
         </is>
       </c>
       <c r="E43" s="34" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="F43" s="37" t="n">
-        <v>0.05</v>
+        <v>4</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H43" s="39" t="inlineStr">
         <is>
-          <t>AliExpress (pack 40)</t>
+          <t>AliExpress</t>
         </is>
       </c>
     </row>
@@ -1933,26 +1933,26 @@
       </c>
       <c r="C44" s="35" t="inlineStr">
         <is>
-          <t>Rallonge capteur JST-XH 3 pins</t>
+          <t>Câbles Dupont F-F 20cm</t>
         </is>
       </c>
       <c r="D44" s="36" t="inlineStr">
         <is>
-          <t>Capteurs déportés</t>
+          <t>MUX ↔ breakout</t>
         </is>
       </c>
       <c r="E44" s="34" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="F44" s="37" t="n">
-        <v>0.8</v>
+        <v>0.05</v>
       </c>
       <c r="G44" s="38" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="H44" s="39" t="inlineStr">
         <is>
-          <t>AliExpress (lot 10)</t>
+          <t>AliExpress (pack 40)</t>
         </is>
       </c>
     </row>
@@ -1967,26 +1967,26 @@
       </c>
       <c r="C45" s="35" t="inlineStr">
         <is>
-          <t>Gaine thermorétractable</t>
+          <t>Rallonge capteur JST-XH 3 pins</t>
         </is>
       </c>
       <c r="D45" s="36" t="inlineStr">
         <is>
-          <t>2-10mm, protection</t>
+          <t>Capteurs déportés</t>
         </is>
       </c>
       <c r="E45" s="34" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F45" s="37" t="n">
-        <v>3</v>
+        <v>0.8</v>
       </c>
       <c r="G45" s="38" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H45" s="39" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>AliExpress (lot 10)</t>
         </is>
       </c>
     </row>
@@ -2001,92 +2001,92 @@
       </c>
       <c r="C46" s="35" t="inlineStr">
         <is>
-          <t>Serre-câbles nylon 100mm</t>
+          <t>Gaine thermorétractable</t>
         </is>
       </c>
       <c r="D46" s="36" t="inlineStr">
         <is>
-          <t>Gestion câbles</t>
+          <t>2-10mm, protection</t>
         </is>
       </c>
       <c r="E46" s="34" t="n">
         <v>1</v>
       </c>
       <c r="F46" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G46" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="H46" s="39" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="15" customHeight="1" s="27">
+      <c r="A47" s="34" t="n">
+        <v>36</v>
+      </c>
+      <c r="B47" s="35" t="inlineStr">
+        <is>
+          <t>CÂBLAGE PLUG-AND-PLAY</t>
+        </is>
+      </c>
+      <c r="C47" s="35" t="inlineStr">
+        <is>
+          <t>Serre-câbles nylon 100mm</t>
+        </is>
+      </c>
+      <c r="D47" s="36" t="inlineStr">
+        <is>
+          <t>Gestion câbles</t>
+        </is>
+      </c>
+      <c r="E47" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F47" s="37" t="n">
         <v>2</v>
       </c>
-      <c r="G46" s="38" t="n">
+      <c r="G47" s="38" t="n">
         <v>2</v>
       </c>
-      <c r="H46" s="39" t="inlineStr">
+      <c r="H47" s="39" t="inlineStr">
         <is>
           <t>Bricomarché (lot 100)</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="15" customHeight="1" s="27">
-      <c r="A47" s="41" t="inlineStr">
+    <row r="48" ht="15" customHeight="1" s="27">
+      <c r="A48" s="41" t="inlineStr">
         <is>
           <t>Sous-total CÂBLAGE PLUG-AND-PLAY</t>
-        </is>
-      </c>
-      <c r="B47" s="32" t="n"/>
-      <c r="C47" s="32" t="n"/>
-      <c r="D47" s="32" t="n"/>
-      <c r="E47" s="32" t="n"/>
-      <c r="F47" s="33" t="n"/>
-      <c r="G47" s="42" t="n">
-        <v>34</v>
-      </c>
-      <c r="H47" s="43" t="n"/>
-    </row>
-    <row r="48" ht="15" customHeight="1" s="27">
-      <c r="A48" s="31" t="inlineStr">
-        <is>
-          <t>📦 BOÎTIER MAÎTRE (intérieur)</t>
         </is>
       </c>
       <c r="B48" s="32" t="n"/>
       <c r="C48" s="32" t="n"/>
       <c r="D48" s="32" t="n"/>
       <c r="E48" s="32" t="n"/>
-      <c r="F48" s="32" t="n"/>
-      <c r="G48" s="32" t="n"/>
-      <c r="H48" s="33" t="n"/>
+      <c r="F48" s="33" t="n"/>
+      <c r="G48" s="42" t="n">
+        <v>34</v>
+      </c>
+      <c r="H48" s="43" t="n"/>
     </row>
     <row r="49" ht="15" customHeight="1" s="27">
-      <c r="A49" s="34" t="n">
-        <v>36</v>
-      </c>
-      <c r="B49" s="35" t="inlineStr">
-        <is>
-          <t>BOÎTIER MAÎTRE (intéri</t>
-        </is>
-      </c>
-      <c r="C49" s="35" t="inlineStr">
-        <is>
-          <t>Boîtier ABS intérieur</t>
-        </is>
-      </c>
-      <c r="D49" s="36" t="inlineStr">
-        <is>
-          <t>200×150×85mm. Pas besoin IP65</t>
-        </is>
-      </c>
-      <c r="E49" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="37" t="n">
-        <v>8</v>
-      </c>
-      <c r="G49" s="38" t="n">
-        <v>8</v>
-      </c>
-      <c r="H49" s="39" t="inlineStr">
-        <is>
-          <t>AliExpress</t>
-        </is>
-      </c>
+      <c r="A49" s="31" t="inlineStr">
+        <is>
+          <t>📦 BOÎTIER MAÎTRE (intérieur)</t>
+        </is>
+      </c>
+      <c r="B49" s="32" t="n"/>
+      <c r="C49" s="32" t="n"/>
+      <c r="D49" s="32" t="n"/>
+      <c r="E49" s="32" t="n"/>
+      <c r="F49" s="32" t="n"/>
+      <c r="G49" s="32" t="n"/>
+      <c r="H49" s="33" t="n"/>
     </row>
     <row r="50" ht="15" customHeight="1" s="27">
       <c r="A50" s="34" t="n">
@@ -2099,22 +2099,22 @@
       </c>
       <c r="C50" s="35" t="inlineStr">
         <is>
-          <t>Bouton poussoir étanche IP67</t>
+          <t>Boîtier ABS intérieur</t>
         </is>
       </c>
       <c r="D50" s="36" t="inlineStr">
         <is>
-          <t>Momentané NO, métal 12mm</t>
+          <t>200×150×85mm. Pas besoin IP65</t>
         </is>
       </c>
       <c r="E50" s="34" t="n">
         <v>1</v>
       </c>
       <c r="F50" s="37" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="G50" s="38" t="n">
-        <v>2.5</v>
+        <v>8</v>
       </c>
       <c r="H50" s="39" t="inlineStr">
         <is>
@@ -2133,22 +2133,22 @@
       </c>
       <c r="C51" s="35" t="inlineStr">
         <is>
-          <t>Plaque support perforée + vis M3</t>
+          <t>Bouton poussoir étanche IP67</t>
         </is>
       </c>
       <c r="D51" s="36" t="inlineStr">
         <is>
-          <t>Fixation ESP32 + modules</t>
+          <t>Momentané NO, métal 12mm</t>
         </is>
       </c>
       <c r="E51" s="34" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="37" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="G51" s="38" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="H51" s="39" t="inlineStr">
         <is>
@@ -2167,92 +2167,92 @@
       </c>
       <c r="C52" s="35" t="inlineStr">
         <is>
-          <t>Entretoises nylon M3</t>
+          <t>Plaque support perforée + vis M3</t>
         </is>
       </c>
       <c r="D52" s="36" t="inlineStr">
         <is>
-          <t>Isolation PCB</t>
+          <t>Fixation ESP32 + modules</t>
         </is>
       </c>
       <c r="E52" s="34" t="n">
         <v>1</v>
       </c>
       <c r="F52" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="39" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="15" customHeight="1" s="27">
+      <c r="A53" s="34" t="n">
+        <v>40</v>
+      </c>
+      <c r="B53" s="35" t="inlineStr">
+        <is>
+          <t>BOÎTIER MAÎTRE (intéri</t>
+        </is>
+      </c>
+      <c r="C53" s="35" t="inlineStr">
+        <is>
+          <t>Entretoises nylon M3</t>
+        </is>
+      </c>
+      <c r="D53" s="36" t="inlineStr">
+        <is>
+          <t>Isolation PCB</t>
+        </is>
+      </c>
+      <c r="E53" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="37" t="n">
         <v>2.5</v>
       </c>
-      <c r="G52" s="38" t="n">
+      <c r="G53" s="38" t="n">
         <v>2.5</v>
       </c>
-      <c r="H52" s="39" t="inlineStr">
+      <c r="H53" s="39" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="15" customHeight="1" s="27">
-      <c r="A53" s="41" t="inlineStr">
+    <row r="54" ht="15" customHeight="1" s="27">
+      <c r="A54" s="41" t="inlineStr">
         <is>
           <t>Sous-total BOÎTIER MAÎTRE (intérieur)</t>
-        </is>
-      </c>
-      <c r="B53" s="32" t="n"/>
-      <c r="C53" s="32" t="n"/>
-      <c r="D53" s="32" t="n"/>
-      <c r="E53" s="32" t="n"/>
-      <c r="F53" s="33" t="n"/>
-      <c r="G53" s="42" t="n">
-        <v>16</v>
-      </c>
-      <c r="H53" s="43" t="n"/>
-    </row>
-    <row r="54" ht="15" customHeight="1" s="27">
-      <c r="A54" s="31" t="inlineStr">
-        <is>
-          <t>📦 BOÎTIER ESCLAVE (balcon IP65)</t>
         </is>
       </c>
       <c r="B54" s="32" t="n"/>
       <c r="C54" s="32" t="n"/>
       <c r="D54" s="32" t="n"/>
       <c r="E54" s="32" t="n"/>
-      <c r="F54" s="32" t="n"/>
-      <c r="G54" s="32" t="n"/>
-      <c r="H54" s="33" t="n"/>
+      <c r="F54" s="33" t="n"/>
+      <c r="G54" s="42" t="n">
+        <v>16</v>
+      </c>
+      <c r="H54" s="43" t="n"/>
     </row>
     <row r="55" ht="15" customHeight="1" s="27">
-      <c r="A55" s="34" t="n">
-        <v>40</v>
-      </c>
-      <c r="B55" s="35" t="inlineStr">
-        <is>
-          <t>BOÎTIER ESCLAVE (balco</t>
-        </is>
-      </c>
-      <c r="C55" s="35" t="inlineStr">
-        <is>
-          <t>Boîtier IP65 ABS BLANC</t>
-        </is>
-      </c>
-      <c r="D55" s="36" t="inlineStr">
-        <is>
-          <t>200×150×85mm, étanche, vis inox</t>
-        </is>
-      </c>
-      <c r="E55" s="34" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="37" t="n">
-        <v>12</v>
-      </c>
-      <c r="G55" s="38" t="n">
-        <v>12</v>
-      </c>
-      <c r="H55" s="39" t="inlineStr">
-        <is>
-          <t>AliExpress — BLANC</t>
-        </is>
-      </c>
+      <c r="A55" s="31" t="inlineStr">
+        <is>
+          <t>📦 BOÎTIER ESCLAVE (balcon IP65)</t>
+        </is>
+      </c>
+      <c r="B55" s="32" t="n"/>
+      <c r="C55" s="32" t="n"/>
+      <c r="D55" s="32" t="n"/>
+      <c r="E55" s="32" t="n"/>
+      <c r="F55" s="32" t="n"/>
+      <c r="G55" s="32" t="n"/>
+      <c r="H55" s="33" t="n"/>
     </row>
     <row r="56" ht="15" customHeight="1" s="27">
       <c r="A56" s="34" t="n">
@@ -2265,26 +2265,26 @@
       </c>
       <c r="C56" s="35" t="inlineStr">
         <is>
-          <t>Presse-étoupe PG7</t>
+          <t>Boîtier IP65 ABS BLANC</t>
         </is>
       </c>
       <c r="D56" s="36" t="inlineStr">
         <is>
-          <t>Câbles capteurs 3-6mm</t>
+          <t>200×150×85mm, étanche, vis inox</t>
         </is>
       </c>
       <c r="E56" s="34" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F56" s="37" t="n">
-        <v>0.5</v>
+        <v>12</v>
       </c>
       <c r="G56" s="38" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="H56" s="39" t="inlineStr">
         <is>
-          <t>AliExpress</t>
+          <t>AliExpress — BLANC</t>
         </is>
       </c>
     </row>
@@ -2299,22 +2299,22 @@
       </c>
       <c r="C57" s="35" t="inlineStr">
         <is>
-          <t>Presse-étoupe PG9</t>
+          <t>Presse-étoupe PG7</t>
         </is>
       </c>
       <c r="D57" s="36" t="inlineStr">
         <is>
-          <t>Câbles puissance 6-8mm</t>
+          <t>Câbles capteurs 3-6mm</t>
         </is>
       </c>
       <c r="E57" s="34" t="n">
+        <v>8</v>
+      </c>
+      <c r="F57" s="37" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G57" s="38" t="n">
         <v>4</v>
-      </c>
-      <c r="F57" s="37" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="G57" s="38" t="n">
-        <v>2.4</v>
       </c>
       <c r="H57" s="39" t="inlineStr">
         <is>
@@ -2333,126 +2333,160 @@
       </c>
       <c r="C58" s="35" t="inlineStr">
         <is>
+          <t>Presse-étoupe PG9</t>
+        </is>
+      </c>
+      <c r="D58" s="36" t="inlineStr">
+        <is>
+          <t>Câbles puissance 6-8mm</t>
+        </is>
+      </c>
+      <c r="E58" s="34" t="n">
+        <v>4</v>
+      </c>
+      <c r="F58" s="37" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G58" s="38" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="H58" s="39" t="inlineStr">
+        <is>
+          <t>AliExpress</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="15" customHeight="1" s="27">
+      <c r="A59" s="34" t="n">
+        <v>44</v>
+      </c>
+      <c r="B59" s="35" t="inlineStr">
+        <is>
+          <t>BOÎTIER ESCLAVE (balco</t>
+        </is>
+      </c>
+      <c r="C59" s="35" t="inlineStr">
+        <is>
           <t>Presse-étoupe PG11</t>
         </is>
       </c>
-      <c r="D58" s="36" t="inlineStr">
+      <c r="D59" s="36" t="inlineStr">
         <is>
           <t>Câble USB + pompe</t>
         </is>
       </c>
-      <c r="E58" s="34" t="n">
+      <c r="E59" s="34" t="n">
         <v>2</v>
       </c>
-      <c r="F58" s="37" t="n">
+      <c r="F59" s="37" t="n">
         <v>0.7</v>
       </c>
-      <c r="G58" s="38" t="n">
+      <c r="G59" s="38" t="n">
         <v>1.4</v>
       </c>
-      <c r="H58" s="39" t="inlineStr">
+      <c r="H59" s="39" t="inlineStr">
         <is>
           <t>AliExpress</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="15" customHeight="1" s="27">
-      <c r="A59" s="41" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="41" t="inlineStr">
         <is>
           <t>Sous-total BOÎTIER ESCLAVE (balcon IP65)</t>
         </is>
       </c>
-      <c r="B59" s="32" t="n"/>
-      <c r="C59" s="32" t="n"/>
-      <c r="D59" s="32" t="n"/>
-      <c r="E59" s="32" t="n"/>
-      <c r="F59" s="33" t="n"/>
-      <c r="G59" s="42" t="n">
+      <c r="B60" s="32" t="n"/>
+      <c r="C60" s="32" t="n"/>
+      <c r="D60" s="32" t="n"/>
+      <c r="E60" s="32" t="n"/>
+      <c r="F60" s="33" t="n"/>
+      <c r="G60" s="42" t="n">
         <v>19.8</v>
       </c>
-      <c r="H59" s="43" t="n"/>
-    </row>
-    <row r="60"/>
-    <row r="61" ht="15" customHeight="1" s="27">
-      <c r="A61" s="45" t="inlineStr">
+      <c r="H60" s="43" t="n"/>
+    </row>
+    <row r="61" ht="15" customHeight="1" s="27"/>
+    <row r="62" ht="15" customHeight="1" s="27">
+      <c r="A62" s="45" t="inlineStr">
         <is>
           <t>TOTAL BOM</t>
         </is>
       </c>
-      <c r="B61" s="32" t="n"/>
-      <c r="C61" s="32" t="n"/>
-      <c r="D61" s="32" t="n"/>
-      <c r="E61" s="32" t="n"/>
-      <c r="F61" s="33" t="n"/>
-      <c r="G61" s="46" t="n">
-        <v>204.4</v>
-      </c>
-      <c r="H61" s="47" t="n"/>
-    </row>
-    <row r="62" ht="15" customHeight="1" s="27">
-      <c r="A62" s="48" t="inlineStr">
+      <c r="B62" s="32" t="n"/>
+      <c r="C62" s="32" t="n"/>
+      <c r="D62" s="32" t="n"/>
+      <c r="E62" s="32" t="n"/>
+      <c r="F62" s="33" t="n"/>
+      <c r="G62" s="46" t="n">
+        <v>214.4</v>
+      </c>
+      <c r="H62" s="47" t="n"/>
+    </row>
+    <row r="63" ht="16.15" customHeight="1" s="27">
+      <c r="A63" s="48" t="inlineStr">
         <is>
           <t>+ Marge rechange 15%</t>
         </is>
       </c>
-      <c r="G62" s="49" t="n">
-        <v>30.66</v>
-      </c>
-    </row>
-    <row r="63" ht="16.15" customHeight="1" s="27">
-      <c r="A63" s="50" t="inlineStr">
+      <c r="G63" s="49" t="n">
+        <v>32.16</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="50" t="inlineStr">
         <is>
           <t>BUDGET TOTAL PROJET</t>
         </is>
       </c>
-      <c r="B63" s="32" t="n"/>
-      <c r="C63" s="32" t="n"/>
-      <c r="D63" s="32" t="n"/>
-      <c r="E63" s="32" t="n"/>
-      <c r="F63" s="33" t="n"/>
-      <c r="G63" s="51" t="n">
-        <v>235.06</v>
-      </c>
-      <c r="H63" s="52" t="n"/>
-    </row>
-    <row r="64"/>
-    <row r="65" ht="15" customHeight="1" s="27">
-      <c r="A65" s="53" t="inlineStr">
+      <c r="B64" s="32" t="n"/>
+      <c r="C64" s="32" t="n"/>
+      <c r="D64" s="32" t="n"/>
+      <c r="E64" s="32" t="n"/>
+      <c r="F64" s="33" t="n"/>
+      <c r="G64" s="51" t="n">
+        <v>246.56</v>
+      </c>
+      <c r="H64" s="52" t="n"/>
+    </row>
+    <row r="65" ht="15" customHeight="1" s="27"/>
+    <row r="66" ht="15" customHeight="1" s="27">
+      <c r="A66" s="53" t="inlineStr">
         <is>
           <t>NOTES:</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="15" customHeight="1" s="27">
-      <c r="A66" s="54" t="inlineStr">
-        <is>
-          <t>• PLUG-AND-PLAY : Aucune soudure. Borniers à vis, Wago 221, Dupont, JST.</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="27">
       <c r="A67" s="54" t="inlineStr">
         <is>
-          <t>• 2× USB SECTEUR : Prise balcon + prise intérieur. Pas de solaire/batterie.</t>
+          <t>• PLUG-AND-PLAY : Aucune soudure. Borniers à vis, Wago 221, Dupont, JST.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="27">
       <c r="A68" s="54" t="inlineStr">
         <is>
-          <t>• SUPPRIMÉ vs v3 : Panneau solaire, MPPT, LiFePO4, LM2596, fusible 5A/thermique, boîtier énergie.</t>
+          <t>• 2× USB SECTEUR : Prise balcon + prise intérieur. Pas de solaire/batterie.</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="27">
       <c r="A69" s="54" t="inlineStr">
         <is>
-          <t>• ÉCONOMIE : ~104€ économisés grâce à la prise secteur balcon.</t>
+          <t>• SUPPRIMÉ vs v3 : Panneau solaire, MPPT, LiFePO4, LM2596, fusible 5A/thermique, boîtier énergie.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="27">
       <c r="A70" s="54" t="inlineStr">
+        <is>
+          <t>• ÉCONOMIE : ~104€ économisés grâce à la prise secteur balcon.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="54" t="inlineStr">
         <is>
           <t>• Zéro gestion thermique batterie — le risque principal du projet est éliminé.</t>
         </is>

</xml_diff>